<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@2b4840e344ec97eadf64b8ede0ae430dfc8916e4 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-bronsysteem-zorgaanbieder.xlsx
+++ b/CodeSystem-bronsysteem-zorgaanbieder.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="57">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-03-04T08:15:04+00:00</t>
+    <t>2024-03-06T08:54:43+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -178,6 +178,12 @@
   </si>
   <si>
     <t>Martini OID</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.4.3.213</t>
+  </si>
+  <si>
+    <t>RIVO-Noord OID</t>
   </si>
 </sst>
 </file>
@@ -493,7 +499,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -594,6 +600,18 @@
       </c>
       <c r="D8" s="2"/>
     </row>
+    <row r="9">
+      <c r="A9" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B9" t="s" s="2">
+        <v>55</v>
+      </c>
+      <c r="C9" t="s" s="2">
+        <v>56</v>
+      </c>
+      <c r="D9" s="2"/>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@838f69c79937d94bbab4feb0983ba0b77b9d97de 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-bronsysteem-zorgaanbieder.xlsx
+++ b/CodeSystem-bronsysteem-zorgaanbieder.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="60">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-04-17T15:52:58+00:00</t>
+    <t>2024-04-17T16:03:08+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -139,6 +139,12 @@
   </si>
   <si>
     <t>1</t>
+  </si>
+  <si>
+    <t>urn:oid:2.16.840.1.113883.2.4.3.98</t>
+  </si>
+  <si>
+    <t>Ommelander Ziekenhuis Groep locatie Delfzicht OID</t>
   </si>
   <si>
     <t>urn:oid:2.16.840.1.113883.2.4.3.8</t>
@@ -502,7 +508,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -615,6 +621,18 @@
       </c>
       <c r="D9" s="2"/>
     </row>
+    <row r="10">
+      <c r="A10" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="B10" t="s" s="2">
+        <v>58</v>
+      </c>
+      <c r="C10" t="s" s="2">
+        <v>59</v>
+      </c>
+      <c r="D10" s="2"/>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@4d5a71cce2539b1f1d85c94e355dca7f5fa47406 🚀
</commit_message>
<xml_diff>
--- a/CodeSystem-bronsysteem-zorgaanbieder.xlsx
+++ b/CodeSystem-bronsysteem-zorgaanbieder.xlsx
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>http://hl7.nl/fhir/zorgviewer/CodeSystem/bronsysteem-zorgaanbieder</t>
+    <t>http://fhir.hl7.nl/zorgviewer/CodeSystem/bronsysteem-zorgaanbieder</t>
   </si>
   <si>
     <t>Version</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-12-18T07:23:17+00:00</t>
+    <t>2024-12-23T09:34:32+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>